<commit_message>
Plots and figures for paper
</commit_message>
<xml_diff>
--- a/rcg/results/Experiment Results.xlsx
+++ b/rcg/results/Experiment Results.xlsx
@@ -1120,13 +1120,13 @@
         <v>1</v>
       </c>
       <c r="O3" s="11">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="P3" s="12">
         <v>0</v>
       </c>
       <c r="Q3" s="15">
-        <v>13.1696181999999</v>
+        <v>16.2324302</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -1179,7 +1179,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="15">
-        <v>3.7777316</v>
+        <v>3.9898094</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -1223,16 +1223,16 @@
         <v>1.6352178</v>
       </c>
       <c r="N5" s="13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="O5" s="11">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="P5" s="12">
         <v>0</v>
       </c>
       <c r="Q5" s="15">
-        <v>16.8762934</v>
+        <v>17.5682384</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -1279,13 +1279,13 @@
         <v>1</v>
       </c>
       <c r="O6" s="11">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="P6" s="12">
         <v>0</v>
       </c>
       <c r="Q6" s="15">
-        <v>34.2228865999999</v>
+        <v>27.392125</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1338,7 +1338,7 @@
         <v>0.4</v>
       </c>
       <c r="Q7" s="15">
-        <v>4.250221</v>
+        <v>4.6724786</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
         <v>0.0666666666666666</v>
       </c>
       <c r="Q8" s="15">
-        <v>56.2399748</v>
+        <v>57.1393512</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1435,16 +1435,16 @@
         <v>10.2997624</v>
       </c>
       <c r="N9" s="13">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="O9" s="11">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="12">
-        <v>0.0666666666666666</v>
+        <v>0.133333333333333</v>
       </c>
       <c r="Q9" s="15">
-        <v>79.5064712</v>
+        <v>40.4729442</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -1488,16 +1488,16 @@
         <v>20.1854934</v>
       </c>
       <c r="N10" s="13">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="O10" s="11">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="P10" s="12">
-        <v>0.466666666666666</v>
+        <v>0.666666666666666</v>
       </c>
       <c r="Q10" s="15">
-        <v>41.956356</v>
+        <v>24.9147764</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
@@ -1541,16 +1541,16 @@
         <v>6.950657</v>
       </c>
       <c r="N11" s="13">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="O11" s="11">
-        <v>1.75</v>
+        <v>1.5</v>
       </c>
       <c r="P11" s="12">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="15">
-        <v>53.771264</v>
+        <v>17.1526375</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
@@ -1594,16 +1594,16 @@
         <v>15.4319575999999</v>
       </c>
       <c r="N12" s="13">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O12" s="11">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="P12" s="12">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="15">
-        <v>43.2523595</v>
+        <v>12.680725</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -1647,16 +1647,16 @@
         <v>12.9844282</v>
       </c>
       <c r="N13" s="13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="O13" s="11">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="P13" s="12">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="15">
-        <v>25.3052864</v>
+        <v>26.6905472</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
@@ -1700,7 +1700,7 @@
         <v>11.2353856</v>
       </c>
       <c r="N14" s="13">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="O14" s="11">
         <v>2.6</v>
@@ -1709,7 +1709,7 @@
         <v>0.266666666666666</v>
       </c>
       <c r="Q14" s="15">
-        <v>41.0777351999999</v>
+        <v>29.3770468</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
@@ -1756,13 +1756,13 @@
         <v>1</v>
       </c>
       <c r="O15" s="11">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="P15" s="12">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="15">
-        <v>9.3082836</v>
+        <v>3.5331314</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
@@ -1815,7 +1815,7 @@
         <v>0</v>
       </c>
       <c r="Q16" s="15">
-        <v>22.6193892</v>
+        <v>16.4652662</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
@@ -1868,7 +1868,7 @@
         <v>0</v>
       </c>
       <c r="Q17" s="15">
-        <v>32.8720644</v>
+        <v>26.8634302</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -1921,7 +1921,7 @@
         <v>0.8</v>
       </c>
       <c r="Q18" s="15">
-        <v>87.3995584</v>
+        <v>55.7266466</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
@@ -1968,13 +1968,13 @@
         <v>0.8</v>
       </c>
       <c r="O19" s="11">
-        <v>10.8</v>
+        <v>4.2</v>
       </c>
       <c r="P19" s="12">
-        <v>0.333333333333333</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="15">
-        <v>60.959738</v>
+        <v>53.6598294</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
@@ -2018,16 +2018,16 @@
         <v>7.45827199999999</v>
       </c>
       <c r="N20" s="13">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="O20" s="11">
-        <v>5.33333333333333</v>
+        <v>2.66666666666666</v>
       </c>
       <c r="P20" s="12">
         <v>1</v>
       </c>
       <c r="Q20" s="15">
-        <v>94.4747739999999</v>
+        <v>33.571799</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -2074,13 +2074,13 @@
         <v>0.8</v>
       </c>
       <c r="O21" s="11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P21" s="12">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="Q21" s="15">
-        <v>78.8273032</v>
+        <v>47.8968445</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
@@ -2127,13 +2127,13 @@
         <v>1</v>
       </c>
       <c r="O22" s="11">
-        <v>4.4</v>
+        <v>5</v>
       </c>
       <c r="P22" s="12">
         <v>1</v>
       </c>
       <c r="Q22" s="15">
-        <v>111.0998226</v>
+        <v>55.0222422</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
@@ -2186,7 +2186,7 @@
         <v>0</v>
       </c>
       <c r="Q23" s="24">
-        <v>52.0539126</v>
+        <v>34.7598604</v>
       </c>
       <c r="R23" s="19"/>
       <c r="S23" s="19"/>
@@ -2249,7 +2249,7 @@
         <v>0</v>
       </c>
       <c r="Q24" s="15">
-        <v>41.6895712</v>
+        <v>38.1373332</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="Q25" s="15">
-        <v>44.7150065999999</v>
+        <v>32.5137487999999</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -2349,13 +2349,13 @@
         <v>1</v>
       </c>
       <c r="O26" s="11">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="P26" s="12">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="Q26" s="15">
-        <v>26.0099222</v>
+        <v>40.1060802</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
@@ -2399,16 +2399,16 @@
         <v>12.3812066</v>
       </c>
       <c r="N27" s="13">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="O27" s="11">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="P27" s="12">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="15">
-        <v>36.3463349999999</v>
+        <v>37.779886</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
@@ -2452,16 +2452,16 @@
         <v>7.7444862</v>
       </c>
       <c r="N28" s="13">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="O28" s="11">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="P28" s="12">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="Q28" s="15">
-        <v>20.700997</v>
+        <v>15.1554522</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -2505,16 +2505,16 @@
         <v>13.9691928</v>
       </c>
       <c r="N29" s="13">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="O29" s="11">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="P29" s="12">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="Q29" s="15">
-        <v>105.671597999999</v>
+        <v>57.148527</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
@@ -2561,13 +2561,13 @@
         <v>1</v>
       </c>
       <c r="O30" s="11">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="P30" s="12">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="Q30" s="15">
-        <v>49.235081</v>
+        <v>35.396426</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
@@ -2611,16 +2611,16 @@
         <v>10.2243076</v>
       </c>
       <c r="N31" s="13">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O31" s="11">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="P31" s="12">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="Q31" s="15">
-        <v>43.1189346</v>
+        <v>25.8896056</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
@@ -2664,16 +2664,16 @@
         <v>8.2544104</v>
       </c>
       <c r="N32" s="13">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="O32" s="11">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="P32" s="12">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="Q32" s="15">
-        <v>37.28285175</v>
+        <v>16.6843864</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
@@ -2720,13 +2720,13 @@
         <v>1</v>
       </c>
       <c r="O33" s="11">
-        <v>6.6</v>
+        <v>4.2</v>
       </c>
       <c r="P33" s="12">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q33" s="15">
-        <v>40.7647018</v>
+        <v>23.3389172</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
@@ -2773,13 +2773,13 @@
         <v>1</v>
       </c>
       <c r="O34" s="11">
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="P34" s="12">
-        <v>0</v>
+        <v>0.131666666666666</v>
       </c>
       <c r="Q34" s="15">
-        <v>104.3310075</v>
+        <v>38.0084436</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
@@ -2832,7 +2832,7 @@
         <v>1</v>
       </c>
       <c r="Q35" s="15">
-        <v>55.5809823333333</v>
+        <v>23.0919242</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
@@ -2879,13 +2879,13 @@
         <v>1</v>
       </c>
       <c r="O36" s="11">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="P36" s="12">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q36" s="15">
-        <v>53.1704544</v>
+        <v>31.9375143999999</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
@@ -2932,13 +2932,13 @@
         <v>1</v>
       </c>
       <c r="O37" s="11">
-        <v>5</v>
+        <v>6.6</v>
       </c>
       <c r="P37" s="12">
         <v>0</v>
       </c>
       <c r="Q37" s="15">
-        <v>58.0497966</v>
+        <v>24.5871244</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -2985,13 +2985,13 @@
         <v>1</v>
       </c>
       <c r="O38" s="11">
-        <v>25.8</v>
+        <v>8.4</v>
       </c>
       <c r="P38" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q38" s="15">
-        <v>73.6921041999999</v>
+        <v>22.0246748</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
@@ -3038,13 +3038,13 @@
         <v>1</v>
       </c>
       <c r="O39" s="11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P39" s="12">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q39" s="15">
-        <v>52.9979843999999</v>
+        <v>24.05066</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
@@ -3091,13 +3091,13 @@
         <v>1</v>
       </c>
       <c r="O40" s="11">
-        <v>9</v>
+        <v>6.4</v>
       </c>
       <c r="P40" s="12">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="Q40" s="15">
-        <v>63.949045</v>
+        <v>16.4689854</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
@@ -3144,13 +3144,13 @@
         <v>1</v>
       </c>
       <c r="O41" s="11">
-        <v>10.2</v>
+        <v>6</v>
       </c>
       <c r="P41" s="12">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="Q41" s="15">
-        <v>65.3722708</v>
+        <v>55.4660314</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.25">
@@ -3197,13 +3197,13 @@
         <v>1</v>
       </c>
       <c r="O42" s="11">
-        <v>15</v>
+        <v>5.2</v>
       </c>
       <c r="P42" s="12">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="Q42" s="15">
-        <v>58.3389911999999</v>
+        <v>20.840663</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">

</xml_diff>